<commit_message>
fix: Phase 6 DriveECU/SensorECU 통합 주행 수정
- DriveECU drive.c: IR 센서 방향 반전(D1=우측 기준), 교차로 전체 감지 직진 케이스 추가
- DriveECU main.c: 하드코딩된 버전 문자열 → APP_VERSION/active_slot 사용
- SensorECU main.c: CAN 초기화 결과(ConfigFilter/Start/Notify/State/ESR) 로깅 추가
</commit_message>
<xml_diff>
--- a/docs/부품_구매_목록.xlsx
+++ b/docs/부품_구매_목록.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="197">
   <si>
     <t>전자부품 구매 목록 — BTM-ECU 프로젝트</t>
   </si>
@@ -557,6 +557,9 @@
   </si>
   <si>
     <t>CM4052 / CU301, 블랙 1m</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>M3 알루미늄 서포트 Female 30mm</t>
@@ -609,7 +612,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -622,6 +625,12 @@
       <sz val="14"/>
       <color rgb="FFffffff"/>
       <name val="맑은 고딕"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -787,7 +796,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -795,118 +804,121 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="12" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="5" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="6" applyFont="1" fillId="13" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="7" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="14" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="14" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -1223,12 +1235,12 @@
   <dimension ref="A1:F89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="41" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="42" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="43" width="36.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="43" width="38.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="43" width="40.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="43" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="42" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="43" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="44" width="36.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="44" width="38.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="44" width="40.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="44" width="14.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="30" customFormat="1" s="1">
@@ -1289,7 +1301,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25" customFormat="1" s="1">
       <c r="A6" s="7"/>
       <c r="B6" s="3"/>
       <c r="C6" s="4"/>
@@ -2231,7 +2243,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="20" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A58" s="31" t="s">
         <v>131</v>
       </c>
@@ -2353,7 +2365,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="20" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75" customFormat="1" s="1">
       <c r="A65" s="36" t="s">
         <v>145</v>
       </c>
@@ -2666,7 +2678,9 @@
       <c r="D82" s="39" t="s">
         <v>180</v>
       </c>
-      <c r="E82" s="39"/>
+      <c r="E82" s="41" t="s">
+        <v>181</v>
+      </c>
       <c r="F82" s="40" t="s">
         <v>22</v>
       </c>
@@ -2679,13 +2693,13 @@
         <v>18</v>
       </c>
       <c r="C83" s="39" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D83" s="39" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E83" s="39" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F83" s="40" t="s">
         <v>22</v>
@@ -2699,13 +2713,13 @@
         <v>19</v>
       </c>
       <c r="C84" s="39" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D84" s="39" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E84" s="39" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F84" s="40" t="s">
         <v>22</v>
@@ -2719,11 +2733,11 @@
         <v>20</v>
       </c>
       <c r="C85" s="39" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D85" s="39"/>
       <c r="E85" s="39" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F85" s="40" t="s">
         <v>22</v>
@@ -2737,11 +2751,11 @@
         <v>21</v>
       </c>
       <c r="C86" s="39" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D86" s="39"/>
       <c r="E86" s="39" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F86" s="40" t="s">
         <v>22</v>
@@ -2755,11 +2769,11 @@
         <v>22</v>
       </c>
       <c r="C87" s="39" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D87" s="39"/>
       <c r="E87" s="39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F87" s="40" t="s">
         <v>22</v>
@@ -2773,11 +2787,11 @@
         <v>23</v>
       </c>
       <c r="C88" s="39" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D88" s="39"/>
       <c r="E88" s="39" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F88" s="40" t="s">
         <v>22</v>
@@ -2791,11 +2805,11 @@
         <v>24</v>
       </c>
       <c r="C89" s="39" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D89" s="39"/>
       <c r="E89" s="39" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F89" s="40" t="s">
         <v>22</v>

</xml_diff>